<commit_message>
Se actualiza plnatilla de preactivador
</commit_message>
<xml_diff>
--- a/src/preactivador/preactivador.xlsx
+++ b/src/preactivador/preactivador.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\TeamComunicaciones\automatizadorteam\src\preactivador\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Camilo Jaramillo\source\repos\Team\Pruebas\Poliedro Despliegues\Integrateam\src\preactivador\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{437C3D3F-784D-4A7B-9C81-34E7A88318E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA7F035-6F5F-4D5E-B755-E4D011CED0C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="3015" windowWidth="13005" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Iccid</t>
   </si>
   <si>
-    <t>Nit</t>
+    <t>Documento</t>
+  </si>
+  <si>
+    <t>TipoDoc</t>
   </si>
   <si>
     <t>Cedula</t>
@@ -35,6 +38,18 @@
   </si>
   <si>
     <t>Mensaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 57101602402358561</t>
+  </si>
+  <si>
+    <t>cc</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 57101602508054274</t>
+  </si>
+  <si>
+    <t>nit</t>
   </si>
 </sst>
 </file>
@@ -397,10 +412,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.44140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -415,6 +437,43 @@
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>1128440365</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>1038626820</v>
+      </c>
+      <c r="E2">
+        <v>3102856769</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>900910667</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>1038626820</v>
+      </c>
+      <c r="E3">
+        <v>3102868710</v>
       </c>
     </row>
   </sheetData>

</xml_diff>